<commit_message>
Jour 13 : INDEX et MATCH
</commit_message>
<xml_diff>
--- a/jour-03-tri-filtres/data/student_data_1000.xlsx
+++ b/jour-03-tri-filtres/data/student_data_1000.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdou\OneDrive\Documents\BootcampExcel\excel-bootcamp-30-jours\jour-03-tri-filtres\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9F31D5-7308-4008-A738-0AE9C63011A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F832D14C-BFAC-496F-8617-3A4FF2FD98B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4023,7 +4023,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -4037,6 +4037,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -4085,7 +4086,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>

</xml_diff>